<commit_message>
📊 Horarios actualizados Línea 141 - 4789
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-28.xlsx
+++ b/data/horarios-141-2026-08-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:30:07</t>
+          <t>Última actualización: 13:50:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:30:07</t>
+          <t>13:50:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:59</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,23 +498,873 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:30:07</t>
+          <t>13:50:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>86</v>
+        <v>5</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>14:02</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>14:13</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>86_EST CHICA-ESC AGRARIA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>23</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>28</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>29</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>30</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>31</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>14:29</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>39</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>44</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>14:35</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>45</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>51</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>51</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>14:43</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>53</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>65</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>65</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>71</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>71</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>15:02</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>72</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>76</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>80</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>88</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>89</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>91</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>92</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>15:31</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>101</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>15:33</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>103</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>110</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>15:42</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>112</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>115</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -531,7 +1381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,14 +1394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:30:07</t>
+          <t>Última actualización: 13:50:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -585,23 +1435,148 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:30:07</t>
+          <t>13:50:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>14:06</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>86</v>
+        <v>16</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215D_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>51</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>71</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>80</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>15:40</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>110</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>115</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -618,7 +1593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -631,14 +1606,116 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:30:07</t>
+          <t>Última actualización: 13:50:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>14:09</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>79</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>13:50:10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>15:36</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>106</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4790
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-28.xlsx
+++ b/data/horarios-141-2026-08-28.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:50:10</t>
+          <t>Última actualización: 21:44:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -1365,6 +1365,381 @@
         <v>115</v>
       </c>
       <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>8</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>17</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>22:09</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>25</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>37</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>37</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>22:23</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>39</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>48</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>22:39</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>55</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>22:54</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>70</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>22:58</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>74</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>23:08</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>84</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>23:13</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>89</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>23:23</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>99</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>23:26</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>102</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>23:38</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>114</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1381,7 +1756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1394,14 +1769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:50:10</t>
+          <t>Última actualización: 21:44:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1577,6 +1952,56 @@
         <v>115</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>22:58</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>74</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>23:38</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>114</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1593,7 +2018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1606,14 +2031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:50:10</t>
+          <t>Última actualización: 21:44:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1716,6 +2141,81 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>21:58</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>28</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>21:44:07</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>37</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>